<commit_message>
feat: add channel dashboard and voice data APIs
</commit_message>
<xml_diff>
--- a/web-import-template-v0.1.xlsx
+++ b/web-import-template-v0.1.xlsx
@@ -2183,7 +2183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G284"/>
+  <dimension ref="A1:G290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="8" min="1" max="1"/>
@@ -11681,6 +11681,207 @@
       <c r="G284" t="inlineStr">
         <is>
           <t>PARK_DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>园区档案</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>EPSG:4326</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>园区经度</t>
+        </is>
+      </c>
+      <c r="G285" t="n">
+        <v>125.182</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>园区档案</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>EPSG:4326</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>园区纬度</t>
+        </is>
+      </c>
+      <c r="G286" t="n">
+        <v>44.432</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>门店</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>park_id</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>所属园区编号；有效新门店必须填写</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>PARK-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>门店</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>channel_type</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>TRADITIONAL_STORE/THIRD_SPACE</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>渠道分类；有效新门店必须填写</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>THIRD_SPACE</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>门店</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>reporting_authorized</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>是否允许 B02 上报经营日报</t>
+        </is>
+      </c>
+      <c r="G289" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>门店</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>公开大屏城市标签</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>长春</t>
         </is>
       </c>
     </row>
@@ -12162,7 +12363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="8" min="1" max="1"/>
@@ -13268,6 +13469,50 @@
       <c r="D50" t="inlineStr">
         <is>
           <t>不纳入集中采购分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>channel_type</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>TRADITIONAL_STORE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>传统门店</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>传统零售终端</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>channel_type</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>THIRD_SPACE</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>第三空间</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>餐饮、会客厅、主题驿站等体验式终端</t>
         </is>
       </c>
     </row>
@@ -14048,7 +14293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="8" min="1" max="1"/>
@@ -14079,25 +14324,35 @@
       </c>
       <c r="D1" s="28" t="inlineStr">
         <is>
+          <t>longitude</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="G1" s="28" t="inlineStr">
         <is>
           <t>source_system</t>
         </is>
       </c>
-      <c r="F1" s="28" t="inlineStr">
+      <c r="H1" s="28" t="inlineStr">
         <is>
           <t>source_record_id</t>
         </is>
       </c>
-      <c r="G1" s="28" t="inlineStr">
+      <c r="I1" s="28" t="inlineStr">
         <is>
           <t>source_updated_at</t>
         </is>
       </c>
-      <c r="H1" s="28" t="inlineStr">
+      <c r="J1" s="28" t="inlineStr">
         <is>
           <t>remark</t>
         </is>
@@ -14115,27 +14370,27 @@
         </is>
       </c>
       <c r="C2" s="23" t="str"/>
-      <c r="D2" s="23" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="E2" s="23" t="inlineStr">
+      <c r="G2" s="23" t="inlineStr">
         <is>
           <t>erp_demo</t>
         </is>
       </c>
-      <c r="F2" s="23" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>ERP-000001</t>
         </is>
       </c>
-      <c r="G2" s="23" t="inlineStr">
+      <c r="I2" s="23" t="inlineStr">
         <is>
           <t>&lt;ISO-8601 datetime&gt;</t>
         </is>
       </c>
-      <c r="H2" s="23" t="str"/>
+      <c r="J2" s="23" t="str"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14376,7 +14631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="8" min="1" max="1"/>
@@ -14413,55 +14668,75 @@
       </c>
       <c r="D1" s="28" t="inlineStr">
         <is>
+          <t>park_id</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>channel_type</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>reporting_authorized</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
           <t>store_name</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="H1" s="28" t="inlineStr">
         <is>
           <t>store_contact_name</t>
         </is>
       </c>
-      <c r="F1" s="28" t="inlineStr">
+      <c r="I1" s="28" t="inlineStr">
         <is>
           <t>store_phone</t>
         </is>
       </c>
-      <c r="G1" s="28" t="inlineStr">
+      <c r="J1" s="28" t="inlineStr">
         <is>
           <t>delivery_address</t>
         </is>
       </c>
-      <c r="H1" s="29" t="inlineStr">
+      <c r="K1" s="29" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="L1" s="29" t="inlineStr">
         <is>
           <t>longitude</t>
         </is>
       </c>
-      <c r="I1" s="29" t="inlineStr">
+      <c r="M1" s="29" t="inlineStr">
         <is>
           <t>latitude</t>
         </is>
       </c>
-      <c r="J1" s="28" t="inlineStr">
+      <c r="N1" s="28" t="inlineStr">
         <is>
           <t>relationship_status</t>
         </is>
       </c>
-      <c r="K1" s="28" t="inlineStr">
+      <c r="O1" s="28" t="inlineStr">
         <is>
           <t>source_system</t>
         </is>
       </c>
-      <c r="L1" s="28" t="inlineStr">
+      <c r="P1" s="28" t="inlineStr">
         <is>
           <t>source_record_id</t>
         </is>
       </c>
-      <c r="M1" s="28" t="inlineStr">
+      <c r="Q1" s="28" t="inlineStr">
         <is>
           <t>source_updated_at</t>
         </is>
       </c>
-      <c r="N1" s="28" t="inlineStr">
+      <c r="R1" s="28" t="inlineStr">
         <is>
           <t>remark</t>
         </is>

</xml_diff>